<commit_message>
Update Waldwunder xlsx, remove temp lock file
</commit_message>
<xml_diff>
--- a/Waldwunder/Angabe/Testdaten/Testdaten/Waldwunder.xlsx
+++ b/Waldwunder/Angabe/Testdaten/Testdaten/Waldwunder.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4506"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wegho\Downloads\POS-Matura\Waldwunder\Angabe\Testdaten\Testdaten\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C3DFC47-1AAE-4B1F-8270-23453CB91E94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="120" yWindow="75" windowWidth="12855" windowHeight="7680"/>
+    <workbookView xWindow="14370" yWindow="3195" windowWidth="23100" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -16,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="49">
   <si>
     <t>Waldwunder</t>
   </si>
@@ -157,13 +163,19 @@
   </si>
   <si>
     <t>47.889462, 14.460751</t>
+  </si>
+  <si>
+    <t>13.646679</t>
+  </si>
+  <si>
+    <t>47.562857</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -200,13 +212,21 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Larissa-Design">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Larissa">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -244,7 +264,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Larissa">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -278,6 +298,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -312,9 +333,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Larissa">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -487,9 +509,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F15"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:F20"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="15.42578125" customWidth="1"/>
     <col min="3" max="3" width="19.5703125" customWidth="1"/>
@@ -497,7 +519,7 @@
     <col min="6" max="6" width="20.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B1" t="s">
         <v>0</v>
       </c>
@@ -514,12 +536,12 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:6">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="3" spans="1:6">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>1</v>
       </c>
@@ -539,7 +561,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:6">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2</v>
       </c>
@@ -559,7 +581,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:6">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>3</v>
       </c>
@@ -579,7 +601,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="6" spans="1:6">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>4</v>
       </c>
@@ -599,7 +621,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="7" spans="1:6">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>5</v>
       </c>
@@ -619,7 +641,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="8" spans="1:6">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>6</v>
       </c>
@@ -639,7 +661,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="9" spans="1:6">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>7</v>
       </c>
@@ -659,7 +681,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="10" spans="1:6">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>8</v>
       </c>
@@ -679,12 +701,12 @@
         <v>35</v>
       </c>
     </row>
-    <row r="12" spans="1:6">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="13" spans="1:6">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
         <v>38</v>
       </c>
@@ -701,7 +723,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="14" spans="1:6">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B14" t="s">
         <v>41</v>
       </c>
@@ -718,7 +740,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="15" spans="1:6">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B15" t="s">
         <v>44</v>
       </c>
@@ -733,6 +755,14 @@
       </c>
       <c r="F15" t="s">
         <v>45</v>
+      </c>
+    </row>
+    <row r="20" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C20" t="s">
+        <v>48</v>
+      </c>
+      <c r="D20" t="s">
+        <v>47</v>
       </c>
     </row>
   </sheetData>
@@ -741,18 +771,18 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>